<commit_message>
project_files housekeeping: remove stale dev ontologies, update registry to 82-row version
</commit_message>
<xml_diff>
--- a/project_files/CCO-Domain-Term-Registry.xlsx
+++ b/project_files/CCO-Domain-Term-Registry.xlsx
@@ -19,7 +19,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
+  </numFmts>
   <fonts count="9">
     <font>
       <name val="Calibri"/>
@@ -138,7 +141,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -261,6 +264,20 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="164" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -626,7 +643,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P61"/>
+  <dimension ref="A1:P83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -731,42 +748,42 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="46" t="inlineStr">
+      <c r="A2" s="48" t="inlineStr">
         <is>
           <t>ent00000001</t>
         </is>
       </c>
-      <c r="B2" s="46" t="inlineStr">
+      <c r="B2" s="48" t="inlineStr">
         <is>
           <t>https://purl.org/cco/ent00000001</t>
         </is>
       </c>
-      <c r="C2" s="47" t="inlineStr">
+      <c r="C2" s="49" t="inlineStr">
         <is>
           <t>Full Name</t>
         </is>
       </c>
-      <c r="D2" s="47" t="inlineStr">
+      <c r="D2" s="49" t="inlineStr">
         <is>
           <t>owl:Class</t>
         </is>
       </c>
-      <c r="E2" s="47" t="inlineStr">
+      <c r="E2" s="49" t="inlineStr">
         <is>
           <t>PersonOntology</t>
         </is>
       </c>
-      <c r="F2" s="46" t="inlineStr">
+      <c r="F2" s="48" t="inlineStr">
         <is>
           <t>https://purl.org/cco/person/FullName</t>
         </is>
       </c>
-      <c r="G2" s="47" t="inlineStr">
+      <c r="G2" s="49" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="H2" s="46" t="inlineStr">
+      <c r="H2" s="48" t="inlineStr">
         <is>
           <t>https://purl.org/cco/ont00001461</t>
         </is>
@@ -776,11 +793,9 @@
           <t>A Proper Name that designates a Person using their complete name.</t>
         </is>
       </c>
-      <c r="J2" s="47" t="inlineStr"/>
-      <c r="K2" s="47" t="inlineStr">
-        <is>
-          <t>2026-02-22</t>
-        </is>
+      <c r="J2" s="49" t="inlineStr"/>
+      <c r="K2" s="50" t="n">
+        <v>46135</v>
       </c>
       <c r="L2" s="4" t="inlineStr"/>
       <c r="M2" s="27" t="inlineStr">
@@ -798,49 +813,49 @@
           <t>Register new ent PURL → ontology file</t>
         </is>
       </c>
-      <c r="P2" s="46" t="inlineStr">
+      <c r="P2" s="48" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/ethical-freelancing/EFO/main/ontology/domains/PersonOntology.ttl</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="46" t="inlineStr">
+      <c r="A3" s="48" t="inlineStr">
         <is>
           <t>ent00000002</t>
         </is>
       </c>
-      <c r="B3" s="46" t="inlineStr">
+      <c r="B3" s="48" t="inlineStr">
         <is>
           <t>https://purl.org/cco/ent00000002</t>
         </is>
       </c>
-      <c r="C3" s="47" t="inlineStr">
+      <c r="C3" s="49" t="inlineStr">
         <is>
           <t>Given Name</t>
         </is>
       </c>
-      <c r="D3" s="47" t="inlineStr">
+      <c r="D3" s="49" t="inlineStr">
         <is>
           <t>owl:Class</t>
         </is>
       </c>
-      <c r="E3" s="47" t="inlineStr">
+      <c r="E3" s="49" t="inlineStr">
         <is>
           <t>PersonOntology</t>
         </is>
       </c>
-      <c r="F3" s="46" t="inlineStr">
+      <c r="F3" s="48" t="inlineStr">
         <is>
           <t>https://purl.org/cco/person/GivenName</t>
         </is>
       </c>
-      <c r="G3" s="47" t="inlineStr">
+      <c r="G3" s="49" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="H3" s="46" t="inlineStr">
+      <c r="H3" s="48" t="inlineStr">
         <is>
           <t>https://purl.org/cco/ont00001461</t>
         </is>
@@ -850,11 +865,9 @@
           <t>A Proper Name component designating the given (first) name of a Person.</t>
         </is>
       </c>
-      <c r="J3" s="47" t="inlineStr"/>
-      <c r="K3" s="47" t="inlineStr">
-        <is>
-          <t>2026-02-22</t>
-        </is>
+      <c r="J3" s="49" t="inlineStr"/>
+      <c r="K3" s="50" t="n">
+        <v>46135</v>
       </c>
       <c r="L3" s="4" t="inlineStr"/>
       <c r="M3" s="27" t="inlineStr">
@@ -873,49 +886,49 @@
 2. Update old PURL → redirect to ent IRI</t>
         </is>
       </c>
-      <c r="P3" s="46" t="inlineStr">
+      <c r="P3" s="48" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/ethical-freelancing/EFO/main/ontology/domains/PersonOntology.ttl</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="46" t="inlineStr">
+      <c r="A4" s="48" t="inlineStr">
         <is>
           <t>ent00000003</t>
         </is>
       </c>
-      <c r="B4" s="46" t="inlineStr">
+      <c r="B4" s="48" t="inlineStr">
         <is>
           <t>https://purl.org/cco/ent00000003</t>
         </is>
       </c>
-      <c r="C4" s="47" t="inlineStr">
+      <c r="C4" s="49" t="inlineStr">
         <is>
           <t>Additional Name</t>
         </is>
       </c>
-      <c r="D4" s="47" t="inlineStr">
+      <c r="D4" s="49" t="inlineStr">
         <is>
           <t>owl:Class</t>
         </is>
       </c>
-      <c r="E4" s="47" t="inlineStr">
+      <c r="E4" s="49" t="inlineStr">
         <is>
           <t>PersonOntology</t>
         </is>
       </c>
-      <c r="F4" s="46" t="inlineStr">
+      <c r="F4" s="48" t="inlineStr">
         <is>
           <t>https://purl.org/cco/person/AdditionalName</t>
         </is>
       </c>
-      <c r="G4" s="47" t="inlineStr">
+      <c r="G4" s="49" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="H4" s="46" t="inlineStr">
+      <c r="H4" s="48" t="inlineStr">
         <is>
           <t>https://purl.org/cco/ont00001461</t>
         </is>
@@ -925,11 +938,9 @@
           <t>A Proper Name component designating a middle or additional name of a Person.</t>
         </is>
       </c>
-      <c r="J4" s="47" t="inlineStr"/>
-      <c r="K4" s="47" t="inlineStr">
-        <is>
-          <t>2026-02-22</t>
-        </is>
+      <c r="J4" s="49" t="inlineStr"/>
+      <c r="K4" s="50" t="n">
+        <v>46143</v>
       </c>
       <c r="L4" s="4" t="inlineStr"/>
       <c r="M4" s="27" t="inlineStr">
@@ -948,49 +959,49 @@
 2. Update old PURL → redirect to ent IRI</t>
         </is>
       </c>
-      <c r="P4" s="46" t="inlineStr">
+      <c r="P4" s="48" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/ethical-freelancing/EFO/main/ontology/domains/PersonOntology.ttl</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="46" t="inlineStr">
+      <c r="A5" s="48" t="inlineStr">
         <is>
           <t>ent00000004</t>
         </is>
       </c>
-      <c r="B5" s="46" t="inlineStr">
+      <c r="B5" s="48" t="inlineStr">
         <is>
           <t>https://purl.org/cco/ent00000004</t>
         </is>
       </c>
-      <c r="C5" s="47" t="inlineStr">
+      <c r="C5" s="49" t="inlineStr">
         <is>
           <t>Family Name</t>
         </is>
       </c>
-      <c r="D5" s="47" t="inlineStr">
+      <c r="D5" s="49" t="inlineStr">
         <is>
           <t>owl:Class</t>
         </is>
       </c>
-      <c r="E5" s="47" t="inlineStr">
+      <c r="E5" s="49" t="inlineStr">
         <is>
           <t>PersonOntology</t>
         </is>
       </c>
-      <c r="F5" s="46" t="inlineStr">
+      <c r="F5" s="48" t="inlineStr">
         <is>
           <t>https://purl.org/cco/person/FamilyName</t>
         </is>
       </c>
-      <c r="G5" s="47" t="inlineStr">
+      <c r="G5" s="49" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="H5" s="46" t="inlineStr">
+      <c r="H5" s="48" t="inlineStr">
         <is>
           <t>https://purl.org/cco/ont00001461</t>
         </is>
@@ -1000,11 +1011,9 @@
           <t>A Proper Name component designating the family (last) name of a Person.</t>
         </is>
       </c>
-      <c r="J5" s="47" t="inlineStr"/>
-      <c r="K5" s="47" t="inlineStr">
-        <is>
-          <t>2026-02-22</t>
-        </is>
+      <c r="J5" s="49" t="inlineStr"/>
+      <c r="K5" s="50" t="n">
+        <v>46140</v>
       </c>
       <c r="L5" s="4" t="inlineStr"/>
       <c r="M5" s="27" t="inlineStr">
@@ -1023,49 +1032,49 @@
 2. Update old PURL → redirect to ent IRI</t>
         </is>
       </c>
-      <c r="P5" s="46" t="inlineStr">
+      <c r="P5" s="48" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/ethical-freelancing/EFO/main/ontology/domains/PersonOntology.ttl</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="46" t="inlineStr">
+      <c r="A6" s="48" t="inlineStr">
         <is>
           <t>ent00000005</t>
         </is>
       </c>
-      <c r="B6" s="46" t="inlineStr">
+      <c r="B6" s="48" t="inlineStr">
         <is>
           <t>https://purl.org/cco/ent00000005</t>
         </is>
       </c>
-      <c r="C6" s="47" t="inlineStr">
+      <c r="C6" s="49" t="inlineStr">
         <is>
           <t>Suffix</t>
         </is>
       </c>
-      <c r="D6" s="47" t="inlineStr">
+      <c r="D6" s="49" t="inlineStr">
         <is>
           <t>owl:Class</t>
         </is>
       </c>
-      <c r="E6" s="47" t="inlineStr">
+      <c r="E6" s="49" t="inlineStr">
         <is>
           <t>PersonOntology</t>
         </is>
       </c>
-      <c r="F6" s="46" t="inlineStr">
+      <c r="F6" s="48" t="inlineStr">
         <is>
           <t>https://purl.org/cco/person/Suffix</t>
         </is>
       </c>
-      <c r="G6" s="47" t="inlineStr">
+      <c r="G6" s="49" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="H6" s="46" t="inlineStr">
+      <c r="H6" s="48" t="inlineStr">
         <is>
           <t>https://purl.org/cco/ont00001461</t>
         </is>
@@ -1075,11 +1084,9 @@
           <t>A Proper Name component designating an honorific suffix of a Person (e.g., Jr., PhD).</t>
         </is>
       </c>
-      <c r="J6" s="47" t="inlineStr"/>
-      <c r="K6" s="47" t="inlineStr">
-        <is>
-          <t>2026-02-22</t>
-        </is>
+      <c r="J6" s="49" t="inlineStr"/>
+      <c r="K6" s="50" t="n">
+        <v>46143</v>
       </c>
       <c r="L6" s="4" t="inlineStr"/>
       <c r="M6" s="27" t="inlineStr">
@@ -1098,49 +1105,49 @@
 2. Update old PURL → redirect to ent IRI</t>
         </is>
       </c>
-      <c r="P6" s="46" t="inlineStr">
+      <c r="P6" s="48" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/ethical-freelancing/EFO/main/ontology/domains/PersonOntology.ttl</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="46" t="inlineStr">
+      <c r="A7" s="48" t="inlineStr">
         <is>
           <t>ent00000006</t>
         </is>
       </c>
-      <c r="B7" s="46" t="inlineStr">
+      <c r="B7" s="48" t="inlineStr">
         <is>
           <t>https://purl.org/cco/ent00000006</t>
         </is>
       </c>
-      <c r="C7" s="47" t="inlineStr">
+      <c r="C7" s="49" t="inlineStr">
         <is>
           <t>Alternate Name</t>
         </is>
       </c>
-      <c r="D7" s="47" t="inlineStr">
+      <c r="D7" s="49" t="inlineStr">
         <is>
           <t>owl:Class</t>
         </is>
       </c>
-      <c r="E7" s="47" t="inlineStr">
+      <c r="E7" s="49" t="inlineStr">
         <is>
           <t>PersonOntology</t>
         </is>
       </c>
-      <c r="F7" s="46" t="inlineStr">
+      <c r="F7" s="48" t="inlineStr">
         <is>
           <t>https://purl.org/cco/person/AlternateName</t>
         </is>
       </c>
-      <c r="G7" s="47" t="inlineStr">
+      <c r="G7" s="49" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="H7" s="46" t="inlineStr">
+      <c r="H7" s="48" t="inlineStr">
         <is>
           <t>https://purl.org/cco/ont00001461</t>
         </is>
@@ -1150,11 +1157,9 @@
           <t>A Designative Name that designates a Person by an alias, pseudonym, or stage name.</t>
         </is>
       </c>
-      <c r="J7" s="47" t="inlineStr"/>
-      <c r="K7" s="47" t="inlineStr">
-        <is>
-          <t>2026-02-22</t>
-        </is>
+      <c r="J7" s="49" t="inlineStr"/>
+      <c r="K7" s="50" t="n">
+        <v>46141</v>
       </c>
       <c r="L7" s="4" t="inlineStr"/>
       <c r="M7" s="27" t="inlineStr">
@@ -1173,49 +1178,49 @@
 2. Update old PURL → redirect to ent IRI</t>
         </is>
       </c>
-      <c r="P7" s="46" t="inlineStr">
+      <c r="P7" s="48" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/ethical-freelancing/EFO/main/ontology/domains/PersonOntology.ttl</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="46" t="inlineStr">
+      <c r="A8" s="48" t="inlineStr">
         <is>
           <t>ent00000007</t>
         </is>
       </c>
-      <c r="B8" s="46" t="inlineStr">
+      <c r="B8" s="48" t="inlineStr">
         <is>
           <t>https://purl.org/cco/ent00000007</t>
         </is>
       </c>
-      <c r="C8" s="47" t="inlineStr">
+      <c r="C8" s="49" t="inlineStr">
         <is>
           <t>National Person Identifier</t>
         </is>
       </c>
-      <c r="D8" s="47" t="inlineStr">
+      <c r="D8" s="49" t="inlineStr">
         <is>
           <t>owl:Class</t>
         </is>
       </c>
-      <c r="E8" s="47" t="inlineStr">
+      <c r="E8" s="49" t="inlineStr">
         <is>
           <t>PersonOntology</t>
         </is>
       </c>
-      <c r="F8" s="46" t="inlineStr">
+      <c r="F8" s="48" t="inlineStr">
         <is>
           <t>https://purl.org/cco/person/NationalPersonIdentifier</t>
         </is>
       </c>
-      <c r="G8" s="47" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="H8" s="46" t="inlineStr">
+      <c r="G8" s="49" t="inlineStr">
+        <is>
+          <t>Removed</t>
+        </is>
+      </c>
+      <c r="H8" s="48" t="inlineStr">
         <is>
           <t>https://purl.org/cco/ont00000077</t>
         </is>
@@ -1225,13 +1230,17 @@
           <t>A Code Identifier assigned by a national authority to uniquely identify a Person.</t>
         </is>
       </c>
-      <c r="J8" s="47" t="inlineStr"/>
-      <c r="K8" s="47" t="inlineStr">
+      <c r="J8" s="49" t="inlineStr"/>
+      <c r="K8" s="49" t="inlineStr">
         <is>
           <t>2026-02-22</t>
         </is>
       </c>
-      <c r="L8" s="4" t="inlineStr"/>
+      <c r="L8" s="4" t="inlineStr">
+        <is>
+          <t>Removed from PersonOntology v5-5 (2026-05-05, merged to Main 2026-07-10); SSN reparented to Person Identifier (ent00000062)</t>
+        </is>
+      </c>
       <c r="M8" s="27" t="inlineStr">
         <is>
           <t>https://purl.org/cco/ent00000007</t>
@@ -1248,51 +1257,51 @@
 2. Update old PURL → redirect to ent IRI</t>
         </is>
       </c>
-      <c r="P8" s="46" t="inlineStr">
+      <c r="P8" s="48" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/ethical-freelancing/EFO/main/ontology/domains/PersonOntology.ttl</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="46" t="inlineStr">
+      <c r="A9" s="48" t="inlineStr">
         <is>
           <t>ent00000008</t>
         </is>
       </c>
-      <c r="B9" s="46" t="inlineStr">
+      <c r="B9" s="48" t="inlineStr">
         <is>
           <t>https://purl.org/cco/ent00000008</t>
         </is>
       </c>
-      <c r="C9" s="47" t="inlineStr">
+      <c r="C9" s="49" t="inlineStr">
         <is>
           <t>Social Security Number</t>
         </is>
       </c>
-      <c r="D9" s="47" t="inlineStr">
+      <c r="D9" s="49" t="inlineStr">
         <is>
           <t>owl:Class</t>
         </is>
       </c>
-      <c r="E9" s="47" t="inlineStr">
+      <c r="E9" s="49" t="inlineStr">
         <is>
           <t>PersonOntology</t>
         </is>
       </c>
-      <c r="F9" s="46" t="inlineStr">
+      <c r="F9" s="48" t="inlineStr">
         <is>
           <t>https://purl.org/cco/person/SocialSecurityNumber</t>
         </is>
       </c>
-      <c r="G9" s="47" t="inlineStr">
+      <c r="G9" s="49" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="H9" s="46" t="inlineStr">
-        <is>
-          <t>https://purl.org/cco/ent00000007</t>
+      <c r="H9" s="48" t="inlineStr">
+        <is>
+          <t>https://purl.org/cco/ent00000062</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
@@ -1300,15 +1309,13 @@
           <t>A National Person Identifier assigned by the US Social Security Administration.</t>
         </is>
       </c>
-      <c r="J9" s="47" t="inlineStr"/>
-      <c r="K9" s="47" t="inlineStr">
-        <is>
-          <t>2026-02-22</t>
-        </is>
+      <c r="J9" s="49" t="inlineStr"/>
+      <c r="K9" s="50" t="n">
+        <v>46132</v>
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>subclass of NationalPersonIdentifier</t>
+          <t>subclass of NationalPersonIdentifier; Parent reparented ent00000007 -&gt; ent00000062 (Person Identifier) in v5-5</t>
         </is>
       </c>
       <c r="M9" s="27" t="inlineStr">
@@ -1327,51 +1334,51 @@
 2. Update old PURL → redirect to ent IRI</t>
         </is>
       </c>
-      <c r="P9" s="46" t="inlineStr">
+      <c r="P9" s="48" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/ethical-freelancing/EFO/main/ontology/domains/PersonOntology.ttl</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="46" t="inlineStr">
+      <c r="A10" s="48" t="inlineStr">
         <is>
           <t>ent00000009</t>
         </is>
       </c>
-      <c r="B10" s="46" t="inlineStr">
+      <c r="B10" s="48" t="inlineStr">
         <is>
           <t>https://purl.org/cco/ent00000009</t>
         </is>
       </c>
-      <c r="C10" s="47" t="inlineStr">
+      <c r="C10" s="49" t="inlineStr">
         <is>
           <t>Postal Address</t>
         </is>
       </c>
-      <c r="D10" s="47" t="inlineStr">
+      <c r="D10" s="49" t="inlineStr">
         <is>
           <t>owl:Class</t>
         </is>
       </c>
-      <c r="E10" s="47" t="inlineStr">
-        <is>
-          <t>PostalAddressOntology</t>
-        </is>
-      </c>
-      <c r="F10" s="46" t="inlineStr">
+      <c r="E10" s="49" t="inlineStr">
+        <is>
+          <t>AddressOntology</t>
+        </is>
+      </c>
+      <c r="F10" s="48" t="inlineStr">
         <is>
           <t>https://purl.org/cco/postal-address/PostalAddress</t>
         </is>
       </c>
-      <c r="G10" s="47" t="inlineStr">
+      <c r="G10" s="49" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="H10" s="46" t="inlineStr">
-        <is>
-          <t>https://purl.org/cco/ont00001066</t>
+      <c r="H10" s="48" t="inlineStr">
+        <is>
+          <t>cco:ent00000310</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr">
@@ -1379,11 +1386,9 @@
           <t>A Designative Information Content Entity that designates a location for postal delivery.</t>
         </is>
       </c>
-      <c r="J10" s="47" t="inlineStr"/>
-      <c r="K10" s="47" t="inlineStr">
-        <is>
-          <t>2026-02-22</t>
-        </is>
+      <c r="J10" s="49" t="inlineStr"/>
+      <c r="K10" s="50" t="n">
+        <v>46188</v>
       </c>
       <c r="L10" s="4" t="inlineStr"/>
       <c r="M10" s="27" t="inlineStr">
@@ -1402,51 +1407,51 @@
 2. Update old PURL → redirect to ent IRI</t>
         </is>
       </c>
-      <c r="P10" s="46" t="inlineStr">
+      <c r="P10" s="48" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/ethical-freelancing/EFO/main/ontology/domains/PostalAddressOntology.ttl</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="46" t="inlineStr">
+      <c r="A11" s="48" t="inlineStr">
         <is>
           <t>ent00000010</t>
         </is>
       </c>
-      <c r="B11" s="46" t="inlineStr">
+      <c r="B11" s="48" t="inlineStr">
         <is>
           <t>https://purl.org/cco/ent00000010</t>
         </is>
       </c>
-      <c r="C11" s="47" t="inlineStr">
+      <c r="C11" s="49" t="inlineStr">
         <is>
           <t>US Postal Address</t>
         </is>
       </c>
-      <c r="D11" s="47" t="inlineStr">
+      <c r="D11" s="49" t="inlineStr">
         <is>
           <t>owl:Class</t>
         </is>
       </c>
-      <c r="E11" s="47" t="inlineStr">
-        <is>
-          <t>PostalAddressOntology</t>
-        </is>
-      </c>
-      <c r="F11" s="46" t="inlineStr">
+      <c r="E11" s="49" t="inlineStr">
+        <is>
+          <t>AddressOntology</t>
+        </is>
+      </c>
+      <c r="F11" s="48" t="inlineStr">
         <is>
           <t>https://purl.org/cco/postal-address/USPostalAddress</t>
         </is>
       </c>
-      <c r="G11" s="47" t="inlineStr">
+      <c r="G11" s="49" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="H11" s="46" t="inlineStr">
-        <is>
-          <t>https://purl.org/cco/ent00000009</t>
+      <c r="H11" s="48" t="inlineStr">
+        <is>
+          <t>cco:ent00000310</t>
         </is>
       </c>
       <c r="I11" s="4" t="inlineStr">
@@ -1454,11 +1459,9 @@
           <t>A Postal Address conforming to United States Postal Service format.</t>
         </is>
       </c>
-      <c r="J11" s="47" t="inlineStr"/>
-      <c r="K11" s="47" t="inlineStr">
-        <is>
-          <t>2026-02-22</t>
-        </is>
+      <c r="J11" s="49" t="inlineStr"/>
+      <c r="K11" s="50" t="n">
+        <v>46188</v>
       </c>
       <c r="L11" s="4" t="inlineStr"/>
       <c r="M11" s="27" t="inlineStr">
@@ -1477,51 +1480,51 @@
 2. Update old PURL → redirect to ent IRI</t>
         </is>
       </c>
-      <c r="P11" s="46" t="inlineStr">
+      <c r="P11" s="48" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/ethical-freelancing/EFO/main/ontology/domains/PostalAddressOntology.ttl</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="46" t="inlineStr">
+      <c r="A12" s="48" t="inlineStr">
         <is>
           <t>ent00000011</t>
         </is>
       </c>
-      <c r="B12" s="46" t="inlineStr">
+      <c r="B12" s="48" t="inlineStr">
         <is>
           <t>https://purl.org/cco/ent00000011</t>
         </is>
       </c>
-      <c r="C12" s="47" t="inlineStr">
+      <c r="C12" s="49" t="inlineStr">
         <is>
           <t>Street Address</t>
         </is>
       </c>
-      <c r="D12" s="47" t="inlineStr">
+      <c r="D12" s="49" t="inlineStr">
         <is>
           <t>owl:Class</t>
         </is>
       </c>
-      <c r="E12" s="47" t="inlineStr">
-        <is>
-          <t>PostalAddressOntology</t>
-        </is>
-      </c>
-      <c r="F12" s="46" t="inlineStr">
+      <c r="E12" s="49" t="inlineStr">
+        <is>
+          <t>AddressOntology</t>
+        </is>
+      </c>
+      <c r="F12" s="48" t="inlineStr">
         <is>
           <t>https://purl.org/cco/postal-address/StreetAddress</t>
         </is>
       </c>
-      <c r="G12" s="47" t="inlineStr">
+      <c r="G12" s="49" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="H12" s="46" t="inlineStr">
-        <is>
-          <t>https://purl.org/cco/ent00000009</t>
+      <c r="H12" s="48" t="inlineStr">
+        <is>
+          <t>cco:ent00000312</t>
         </is>
       </c>
       <c r="I12" s="4" t="inlineStr">
@@ -1529,11 +1532,9 @@
           <t>A component of a Postal Address designating the street-level location.</t>
         </is>
       </c>
-      <c r="J12" s="47" t="inlineStr"/>
-      <c r="K12" s="47" t="inlineStr">
-        <is>
-          <t>2026-02-22</t>
-        </is>
+      <c r="J12" s="49" t="inlineStr"/>
+      <c r="K12" s="50" t="n">
+        <v>46188</v>
       </c>
       <c r="L12" s="4" t="inlineStr"/>
       <c r="M12" s="27" t="inlineStr">
@@ -1552,51 +1553,51 @@
 2. Update old PURL → redirect to ent IRI</t>
         </is>
       </c>
-      <c r="P12" s="46" t="inlineStr">
+      <c r="P12" s="48" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/ethical-freelancing/EFO/main/ontology/domains/PostalAddressOntology.ttl</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="46" t="inlineStr">
+      <c r="A13" s="48" t="inlineStr">
         <is>
           <t>ent00000012</t>
         </is>
       </c>
-      <c r="B13" s="46" t="inlineStr">
+      <c r="B13" s="48" t="inlineStr">
         <is>
           <t>https://purl.org/cco/ent00000012</t>
         </is>
       </c>
-      <c r="C13" s="47" t="inlineStr">
-        <is>
-          <t>City Name</t>
-        </is>
-      </c>
-      <c r="D13" s="47" t="inlineStr">
+      <c r="C13" s="49" t="inlineStr">
+        <is>
+          <t>City</t>
+        </is>
+      </c>
+      <c r="D13" s="49" t="inlineStr">
         <is>
           <t>owl:Class</t>
         </is>
       </c>
-      <c r="E13" s="47" t="inlineStr">
-        <is>
-          <t>PostalAddressOntology</t>
-        </is>
-      </c>
-      <c r="F13" s="46" t="inlineStr">
+      <c r="E13" s="49" t="inlineStr">
+        <is>
+          <t>AddressOntology</t>
+        </is>
+      </c>
+      <c r="F13" s="48" t="inlineStr">
         <is>
           <t>https://purl.org/cco/postal-address/CityName</t>
         </is>
       </c>
-      <c r="G13" s="47" t="inlineStr">
+      <c r="G13" s="49" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="H13" s="46" t="inlineStr">
-        <is>
-          <t>https://purl.org/cco/ont00001461</t>
+      <c r="H13" s="48" t="inlineStr">
+        <is>
+          <t>cco:ent00000312</t>
         </is>
       </c>
       <c r="I13" s="4" t="inlineStr">
@@ -1604,11 +1605,9 @@
           <t>A Proper Name that designates a city within a Postal Address.</t>
         </is>
       </c>
-      <c r="J13" s="47" t="inlineStr"/>
-      <c r="K13" s="47" t="inlineStr">
-        <is>
-          <t>2026-02-22</t>
-        </is>
+      <c r="J13" s="49" t="inlineStr"/>
+      <c r="K13" s="50" t="n">
+        <v>46188</v>
       </c>
       <c r="L13" s="4" t="inlineStr"/>
       <c r="M13" s="27" t="inlineStr">
@@ -1627,51 +1626,51 @@
 2. Update old PURL → redirect to ent IRI</t>
         </is>
       </c>
-      <c r="P13" s="46" t="inlineStr">
+      <c r="P13" s="48" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/ethical-freelancing/EFO/main/ontology/domains/PostalAddressOntology.ttl</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="46" t="inlineStr">
+      <c r="A14" s="48" t="inlineStr">
         <is>
           <t>ent00000013</t>
         </is>
       </c>
-      <c r="B14" s="46" t="inlineStr">
+      <c r="B14" s="48" t="inlineStr">
         <is>
           <t>https://purl.org/cco/ent00000013</t>
         </is>
       </c>
-      <c r="C14" s="47" t="inlineStr">
-        <is>
-          <t>State Name</t>
-        </is>
-      </c>
-      <c r="D14" s="47" t="inlineStr">
+      <c r="C14" s="49" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="D14" s="49" t="inlineStr">
         <is>
           <t>owl:Class</t>
         </is>
       </c>
-      <c r="E14" s="47" t="inlineStr">
-        <is>
-          <t>PostalAddressOntology</t>
-        </is>
-      </c>
-      <c r="F14" s="46" t="inlineStr">
+      <c r="E14" s="49" t="inlineStr">
+        <is>
+          <t>AddressOntology</t>
+        </is>
+      </c>
+      <c r="F14" s="48" t="inlineStr">
         <is>
           <t>https://purl.org/cco/postal-address/StateName</t>
         </is>
       </c>
-      <c r="G14" s="47" t="inlineStr">
+      <c r="G14" s="49" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="H14" s="46" t="inlineStr">
-        <is>
-          <t>https://purl.org/cco/ont00001461</t>
+      <c r="H14" s="48" t="inlineStr">
+        <is>
+          <t>cco:ent00000312</t>
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr">
@@ -1679,11 +1678,9 @@
           <t>A Proper Name that designates a state or province within a Postal Address.</t>
         </is>
       </c>
-      <c r="J14" s="47" t="inlineStr"/>
-      <c r="K14" s="47" t="inlineStr">
-        <is>
-          <t>2026-02-22</t>
-        </is>
+      <c r="J14" s="49" t="inlineStr"/>
+      <c r="K14" s="50" t="n">
+        <v>46188</v>
       </c>
       <c r="L14" s="4" t="inlineStr"/>
       <c r="M14" s="27" t="inlineStr">
@@ -1702,51 +1699,51 @@
 2. Update old PURL → redirect to ent IRI</t>
         </is>
       </c>
-      <c r="P14" s="46" t="inlineStr">
+      <c r="P14" s="48" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/ethical-freelancing/EFO/main/ontology/domains/PostalAddressOntology.ttl</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="46" t="inlineStr">
+      <c r="A15" s="48" t="inlineStr">
         <is>
           <t>ent00000014</t>
         </is>
       </c>
-      <c r="B15" s="46" t="inlineStr">
+      <c r="B15" s="48" t="inlineStr">
         <is>
           <t>https://purl.org/cco/ent00000014</t>
         </is>
       </c>
-      <c r="C15" s="47" t="inlineStr">
+      <c r="C15" s="49" t="inlineStr">
         <is>
           <t>Country Name</t>
         </is>
       </c>
-      <c r="D15" s="47" t="inlineStr">
+      <c r="D15" s="49" t="inlineStr">
         <is>
           <t>owl:Class</t>
         </is>
       </c>
-      <c r="E15" s="47" t="inlineStr">
-        <is>
-          <t>PostalAddressOntology</t>
-        </is>
-      </c>
-      <c r="F15" s="46" t="inlineStr">
+      <c r="E15" s="49" t="inlineStr">
+        <is>
+          <t>AddressOntology</t>
+        </is>
+      </c>
+      <c r="F15" s="48" t="inlineStr">
         <is>
           <t>https://purl.org/cco/postal-address/CountryName</t>
         </is>
       </c>
-      <c r="G15" s="47" t="inlineStr">
+      <c r="G15" s="49" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="H15" s="46" t="inlineStr">
-        <is>
-          <t>https://purl.org/cco/ont00001461</t>
+      <c r="H15" s="48" t="inlineStr">
+        <is>
+          <t>cco:ent00000312</t>
         </is>
       </c>
       <c r="I15" s="4" t="inlineStr">
@@ -1754,11 +1751,9 @@
           <t>A Proper Name that designates a country within a Postal Address.</t>
         </is>
       </c>
-      <c r="J15" s="47" t="inlineStr"/>
-      <c r="K15" s="47" t="inlineStr">
-        <is>
-          <t>2026-02-22</t>
-        </is>
+      <c r="J15" s="49" t="inlineStr"/>
+      <c r="K15" s="50" t="n">
+        <v>46209</v>
       </c>
       <c r="L15" s="4" t="inlineStr"/>
       <c r="M15" s="27" t="inlineStr">
@@ -1777,51 +1772,51 @@
 2. Update old PURL → redirect to ent IRI</t>
         </is>
       </c>
-      <c r="P15" s="46" t="inlineStr">
+      <c r="P15" s="48" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/ethical-freelancing/EFO/main/ontology/domains/PostalAddressOntology.ttl</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="46" t="inlineStr">
+      <c r="A16" s="48" t="inlineStr">
         <is>
           <t>ent00000015</t>
         </is>
       </c>
-      <c r="B16" s="46" t="inlineStr">
+      <c r="B16" s="48" t="inlineStr">
         <is>
           <t>https://purl.org/cco/ent00000015</t>
         </is>
       </c>
-      <c r="C16" s="47" t="inlineStr">
+      <c r="C16" s="49" t="inlineStr">
         <is>
           <t>Postal Code</t>
         </is>
       </c>
-      <c r="D16" s="47" t="inlineStr">
+      <c r="D16" s="49" t="inlineStr">
         <is>
           <t>owl:Class</t>
         </is>
       </c>
-      <c r="E16" s="47" t="inlineStr">
-        <is>
-          <t>PostalAddressOntology</t>
-        </is>
-      </c>
-      <c r="F16" s="46" t="inlineStr">
+      <c r="E16" s="49" t="inlineStr">
+        <is>
+          <t>AddressOntology</t>
+        </is>
+      </c>
+      <c r="F16" s="48" t="inlineStr">
         <is>
           <t>https://purl.org/cco/postal-address/PostalCode</t>
         </is>
       </c>
-      <c r="G16" s="47" t="inlineStr">
+      <c r="G16" s="49" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="H16" s="46" t="inlineStr">
-        <is>
-          <t>https://purl.org/cco/ont00000077</t>
+      <c r="H16" s="48" t="inlineStr">
+        <is>
+          <t>cco:ent00000312</t>
         </is>
       </c>
       <c r="I16" s="4" t="inlineStr">
@@ -1829,11 +1824,9 @@
           <t>A Code Identifier designating a postal delivery zone.</t>
         </is>
       </c>
-      <c r="J16" s="47" t="inlineStr"/>
-      <c r="K16" s="47" t="inlineStr">
-        <is>
-          <t>2026-02-22</t>
-        </is>
+      <c r="J16" s="49" t="inlineStr"/>
+      <c r="K16" s="50" t="n">
+        <v>46188</v>
       </c>
       <c r="L16" s="4" t="inlineStr"/>
       <c r="M16" s="27" t="inlineStr">
@@ -1852,49 +1845,49 @@
 2. Update old PURL → redirect to ent IRI</t>
         </is>
       </c>
-      <c r="P16" s="46" t="inlineStr">
+      <c r="P16" s="48" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/ethical-freelancing/EFO/main/ontology/domains/PostalAddressOntology.ttl</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="46" t="inlineStr">
+      <c r="A17" s="48" t="inlineStr">
         <is>
           <t>ent00000016</t>
         </is>
       </c>
-      <c r="B17" s="46" t="inlineStr">
+      <c r="B17" s="48" t="inlineStr">
         <is>
           <t>https://purl.org/cco/ent00000016</t>
         </is>
       </c>
-      <c r="C17" s="47" t="inlineStr">
+      <c r="C17" s="49" t="inlineStr">
         <is>
           <t>Address Designation</t>
         </is>
       </c>
-      <c r="D17" s="47" t="inlineStr">
+      <c r="D17" s="49" t="inlineStr">
         <is>
           <t>owl:Class</t>
         </is>
       </c>
-      <c r="E17" s="47" t="inlineStr">
-        <is>
-          <t>PostalAddressOntology</t>
-        </is>
-      </c>
-      <c r="F17" s="46" t="inlineStr">
+      <c r="E17" s="49" t="inlineStr">
+        <is>
+          <t>AddressOntology</t>
+        </is>
+      </c>
+      <c r="F17" s="48" t="inlineStr">
         <is>
           <t>https://purl.org/cco/postal-address/AddressDesignation</t>
         </is>
       </c>
-      <c r="G17" s="47" t="inlineStr">
+      <c r="G17" s="49" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="H17" s="46" t="inlineStr">
+      <c r="H17" s="48" t="inlineStr">
         <is>
           <t>http://purl.obolibrary.org/obo/BFO_0000015</t>
         </is>
@@ -1904,15 +1897,13 @@
           <t>A Process in which a Person is associated with a Postal Address during a temporal interval.</t>
         </is>
       </c>
-      <c r="J17" s="47" t="inlineStr"/>
-      <c r="K17" s="47" t="inlineStr">
-        <is>
-          <t>2026-02-22</t>
-        </is>
+      <c r="J17" s="49" t="inlineStr"/>
+      <c r="K17" s="50" t="n">
+        <v>46210</v>
       </c>
       <c r="L17" s="4" t="inlineStr">
         <is>
-          <t>Temporal address tracking; BFO Process subclass</t>
+          <t>Temporal address tracking; BFO Process subclass; Re-added to AddressOntology 2026-07-08 (version 2026-07-08); committed to Main 2026-07-09</t>
         </is>
       </c>
       <c r="M17" s="27" t="inlineStr">
@@ -1931,63 +1922,61 @@
 2. Update old PURL → redirect to ent IRI</t>
         </is>
       </c>
-      <c r="P17" s="46" t="inlineStr">
+      <c r="P17" s="48" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/ethical-freelancing/EFO/main/ontology/domains/PostalAddressOntology.ttl</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="46" t="inlineStr">
+      <c r="A18" s="48" t="inlineStr">
         <is>
           <t>ent00000017</t>
         </is>
       </c>
-      <c r="B18" s="46" t="inlineStr">
+      <c r="B18" s="48" t="inlineStr">
         <is>
           <t>https://purl.org/cco/ent00000017</t>
         </is>
       </c>
-      <c r="C18" s="47" t="inlineStr">
+      <c r="C18" s="49" t="inlineStr">
         <is>
           <t>has start date</t>
         </is>
       </c>
-      <c r="D18" s="47" t="inlineStr">
+      <c r="D18" s="49" t="inlineStr">
         <is>
           <t>owl:DatatypeProperty</t>
         </is>
       </c>
-      <c r="E18" s="47" t="inlineStr">
-        <is>
-          <t>PostalAddressOntology</t>
-        </is>
-      </c>
-      <c r="F18" s="46" t="inlineStr">
+      <c r="E18" s="49" t="inlineStr">
+        <is>
+          <t>StagingOntology</t>
+        </is>
+      </c>
+      <c r="F18" s="48" t="inlineStr">
         <is>
           <t>https://purl.org/cco/postal-address/hasStartDate</t>
         </is>
       </c>
-      <c r="G18" s="47" t="inlineStr">
+      <c r="G18" s="49" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="H18" s="46" t="inlineStr"/>
+      <c r="H18" s="48" t="inlineStr"/>
       <c r="I18" s="4" t="inlineStr">
         <is>
           <t>Relates an Address Designation to the date on which it began.</t>
         </is>
       </c>
-      <c r="J18" s="47" t="inlineStr"/>
-      <c r="K18" s="47" t="inlineStr">
-        <is>
-          <t>2026-02-22</t>
-        </is>
+      <c r="J18" s="49" t="inlineStr"/>
+      <c r="K18" s="50" t="n">
+        <v>46212</v>
       </c>
       <c r="L18" s="4" t="inlineStr">
         <is>
-          <t>range: xsd:date</t>
+          <t>range: xsd:date; Relocated from AddressOntology to StagingOntology 2026-07-09 (generic temporal property, not address-specific); IRI unchanged</t>
         </is>
       </c>
       <c r="M18" s="27" t="inlineStr">
@@ -2006,63 +1995,61 @@
 2. Update old PURL → redirect to ent IRI</t>
         </is>
       </c>
-      <c r="P18" s="46" t="inlineStr">
+      <c r="P18" s="48" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/ethical-freelancing/EFO/main/ontology/domains/PostalAddressOntology.ttl</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="46" t="inlineStr">
+      <c r="A19" s="48" t="inlineStr">
         <is>
           <t>ent00000018</t>
         </is>
       </c>
-      <c r="B19" s="46" t="inlineStr">
+      <c r="B19" s="48" t="inlineStr">
         <is>
           <t>https://purl.org/cco/ent00000018</t>
         </is>
       </c>
-      <c r="C19" s="47" t="inlineStr">
+      <c r="C19" s="49" t="inlineStr">
         <is>
           <t>has end date</t>
         </is>
       </c>
-      <c r="D19" s="47" t="inlineStr">
+      <c r="D19" s="49" t="inlineStr">
         <is>
           <t>owl:DatatypeProperty</t>
         </is>
       </c>
-      <c r="E19" s="47" t="inlineStr">
-        <is>
-          <t>PostalAddressOntology</t>
-        </is>
-      </c>
-      <c r="F19" s="46" t="inlineStr">
+      <c r="E19" s="49" t="inlineStr">
+        <is>
+          <t>StagingOntology</t>
+        </is>
+      </c>
+      <c r="F19" s="48" t="inlineStr">
         <is>
           <t>https://purl.org/cco/postal-address/hasEndDate</t>
         </is>
       </c>
-      <c r="G19" s="47" t="inlineStr">
+      <c r="G19" s="49" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="H19" s="46" t="inlineStr"/>
+      <c r="H19" s="48" t="inlineStr"/>
       <c r="I19" s="4" t="inlineStr">
         <is>
           <t>Relates an Address Designation to the date on which it ended; absent if current address.</t>
         </is>
       </c>
-      <c r="J19" s="47" t="inlineStr"/>
-      <c r="K19" s="47" t="inlineStr">
-        <is>
-          <t>2026-02-22</t>
-        </is>
+      <c r="J19" s="49" t="inlineStr"/>
+      <c r="K19" s="50" t="n">
+        <v>46212</v>
       </c>
       <c r="L19" s="4" t="inlineStr">
         <is>
-          <t>range: xsd:date; optional — absence = current</t>
+          <t>range: xsd:date; optional — absence = current; Relocated from AddressOntology to StagingOntology 2026-07-09 (generic temporal property, not address-specific); IRI unchanged</t>
         </is>
       </c>
       <c r="M19" s="27" t="inlineStr">
@@ -2081,7 +2068,7 @@
 2. Update old PURL → redirect to ent IRI</t>
         </is>
       </c>
-      <c r="P19" s="46" t="inlineStr">
+      <c r="P19" s="48" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/ethical-freelancing/EFO/main/ontology/domains/PostalAddressOntology.ttl</t>
         </is>
@@ -2270,7 +2257,7 @@
       </c>
       <c r="G22" s="6" t="inlineStr">
         <is>
-          <t>Infrastructure</t>
+          <t>Retired</t>
         </is>
       </c>
       <c r="H22" s="5" t="inlineStr"/>
@@ -2287,7 +2274,7 @@
       </c>
       <c r="L22" s="7" t="inlineStr">
         <is>
-          <t>Staging infrastructure</t>
+          <t>Staging infrastructure | Property retired 2026-08-04 per DL-015 (superseded by dcterms:created); declaration removed from StagingOntology.ttl.</t>
         </is>
       </c>
       <c r="M22" s="28" t="inlineStr">
@@ -3552,18 +3539,18 @@
       </c>
       <c r="E38" s="35" t="inlineStr">
         <is>
-          <t>persona.ttl (→ PersonOntology on promotion)</t>
+          <t>PersonOntology</t>
         </is>
       </c>
       <c r="F38" s="34" t="inlineStr"/>
       <c r="G38" s="35" t="inlineStr">
         <is>
-          <t>Minted</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="H38" s="34" t="inlineStr">
         <is>
-          <t>https://purl.org/cco/ont00001835</t>
+          <t>https://purl.org/cco/ont00000378  # Color (was ont00001835 'is son of' — ERROR corrected)</t>
         </is>
       </c>
       <c r="I38" s="33" t="inlineStr">
@@ -3576,14 +3563,12 @@
           <t>PersonOntology</t>
         </is>
       </c>
-      <c r="K38" s="35" t="inlineStr">
-        <is>
-          <t>2026-03-17</t>
-        </is>
+      <c r="K38" s="51" t="n">
+        <v>46214</v>
       </c>
       <c r="L38" s="33" t="inlineStr">
         <is>
-          <t>Mint now; currently in persona.ttl</t>
+          <t>Mint now; currently in persona.ttl; Promoted to PersonOntology 2026-07-11 (committed to Main); Option B: closeMatch (not exactMatch) to CCO colors</t>
         </is>
       </c>
       <c r="M38" s="34" t="inlineStr">
@@ -3631,13 +3616,13 @@
       </c>
       <c r="E39" s="35" t="inlineStr">
         <is>
-          <t>persona.ttl (→ PersonOntology on promotion)</t>
+          <t>PersonOntology</t>
         </is>
       </c>
       <c r="F39" s="34" t="inlineStr"/>
       <c r="G39" s="35" t="inlineStr">
         <is>
-          <t>Minted</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="H39" s="34" t="inlineStr">
@@ -3655,14 +3640,12 @@
           <t>PersonOntology</t>
         </is>
       </c>
-      <c r="K39" s="35" t="inlineStr">
-        <is>
-          <t>2026-03-17</t>
-        </is>
+      <c r="K39" s="51" t="n">
+        <v>46214</v>
       </c>
       <c r="L39" s="33" t="inlineStr">
         <is>
-          <t>Property linking Person → EyeColor</t>
+          <t>Property linking Person → EyeColor; Promoted to PersonOntology 2026-07-11 (committed to Main); Option B: closeMatch (not exactMatch) to CCO colors</t>
         </is>
       </c>
       <c r="M39" s="34" t="inlineStr">
@@ -3710,13 +3693,13 @@
       </c>
       <c r="E40" s="35" t="inlineStr">
         <is>
-          <t>persona.ttl (→ PersonOntology on promotion)</t>
+          <t>PersonOntology</t>
         </is>
       </c>
       <c r="F40" s="34" t="inlineStr"/>
       <c r="G40" s="35" t="inlineStr">
         <is>
-          <t>Minted</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="H40" s="34" t="inlineStr">
@@ -3734,14 +3717,12 @@
           <t>PersonOntology</t>
         </is>
       </c>
-      <c r="K40" s="35" t="inlineStr">
-        <is>
-          <t>2026-03-17</t>
-        </is>
+      <c r="K40" s="51" t="n">
+        <v>46214</v>
       </c>
       <c r="L40" s="33" t="inlineStr">
         <is>
-          <t>No CCO color match for amber</t>
+          <t>No CCO color match for amber; Promoted to PersonOntology 2026-07-11 (committed to Main); Option B: closeMatch (not exactMatch) to CCO colors</t>
         </is>
       </c>
       <c r="M40" s="34" t="inlineStr">
@@ -3789,13 +3770,13 @@
       </c>
       <c r="E41" s="35" t="inlineStr">
         <is>
-          <t>persona.ttl (→ PersonOntology on promotion)</t>
+          <t>PersonOntology</t>
         </is>
       </c>
       <c r="F41" s="34" t="inlineStr"/>
       <c r="G41" s="35" t="inlineStr">
         <is>
-          <t>Minted</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="H41" s="34" t="inlineStr">
@@ -3813,14 +3794,12 @@
           <t>PersonOntology</t>
         </is>
       </c>
-      <c r="K41" s="35" t="inlineStr">
-        <is>
-          <t>2026-03-17</t>
-        </is>
+      <c r="K41" s="51" t="n">
+        <v>46214</v>
       </c>
       <c r="L41" s="33" t="inlineStr">
         <is>
-          <t>skos:exactMatch cco:ont00001189</t>
+          <t>skos:exactMatch cco:ont00001189; Promoted to PersonOntology 2026-07-11 (committed to Main); Option B: closeMatch (not exactMatch) to CCO colors</t>
         </is>
       </c>
       <c r="M41" s="34" t="inlineStr">
@@ -3868,13 +3847,13 @@
       </c>
       <c r="E42" s="35" t="inlineStr">
         <is>
-          <t>persona.ttl (→ PersonOntology on promotion)</t>
+          <t>PersonOntology</t>
         </is>
       </c>
       <c r="F42" s="34" t="inlineStr"/>
       <c r="G42" s="35" t="inlineStr">
         <is>
-          <t>Minted</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="H42" s="34" t="inlineStr">
@@ -3892,14 +3871,12 @@
           <t>PersonOntology</t>
         </is>
       </c>
-      <c r="K42" s="35" t="inlineStr">
-        <is>
-          <t>2026-03-17</t>
-        </is>
+      <c r="K42" s="51" t="n">
+        <v>46214</v>
       </c>
       <c r="L42" s="33" t="inlineStr">
         <is>
-          <t>skos:exactMatch cco:ont00000872</t>
+          <t>skos:exactMatch cco:ont00000872; Promoted to PersonOntology 2026-07-11 (committed to Main); Option B: closeMatch (not exactMatch) to CCO colors</t>
         </is>
       </c>
       <c r="M42" s="34" t="inlineStr">
@@ -3937,7 +3914,7 @@
       </c>
       <c r="C43" s="35" t="inlineStr">
         <is>
-          <t>Gray Eye Color</t>
+          <t>Grey Eye Color</t>
         </is>
       </c>
       <c r="D43" s="35" t="inlineStr">
@@ -3947,13 +3924,13 @@
       </c>
       <c r="E43" s="35" t="inlineStr">
         <is>
-          <t>persona.ttl (→ PersonOntology on promotion)</t>
+          <t>PersonOntology</t>
         </is>
       </c>
       <c r="F43" s="34" t="inlineStr"/>
       <c r="G43" s="35" t="inlineStr">
         <is>
-          <t>Minted</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="H43" s="34" t="inlineStr">
@@ -3971,14 +3948,12 @@
           <t>PersonOntology</t>
         </is>
       </c>
-      <c r="K43" s="35" t="inlineStr">
-        <is>
-          <t>2026-03-17</t>
-        </is>
+      <c r="K43" s="51" t="n">
+        <v>46214</v>
       </c>
       <c r="L43" s="33" t="inlineStr">
         <is>
-          <t>skos:exactMatch cco:ont00001349</t>
+          <t>skos:exactMatch cco:ont00001349; Promoted to PersonOntology 2026-07-11 (committed to Main); Option B: closeMatch (not exactMatch) to CCO colors</t>
         </is>
       </c>
       <c r="M43" s="34" t="inlineStr">
@@ -4026,13 +4001,13 @@
       </c>
       <c r="E44" s="35" t="inlineStr">
         <is>
-          <t>persona.ttl (→ PersonOntology on promotion)</t>
+          <t>PersonOntology</t>
         </is>
       </c>
       <c r="F44" s="34" t="inlineStr"/>
       <c r="G44" s="35" t="inlineStr">
         <is>
-          <t>Minted</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="H44" s="34" t="inlineStr">
@@ -4050,14 +4025,12 @@
           <t>PersonOntology</t>
         </is>
       </c>
-      <c r="K44" s="35" t="inlineStr">
-        <is>
-          <t>2026-03-17</t>
-        </is>
+      <c r="K44" s="51" t="n">
+        <v>46214</v>
       </c>
       <c r="L44" s="33" t="inlineStr">
         <is>
-          <t>skos:exactMatch cco:ont00000082</t>
+          <t>skos:exactMatch cco:ont00000082; Promoted to PersonOntology 2026-07-11 (committed to Main); Option B: closeMatch (not exactMatch) to CCO colors</t>
         </is>
       </c>
       <c r="M44" s="34" t="inlineStr">
@@ -4105,13 +4078,13 @@
       </c>
       <c r="E45" s="35" t="inlineStr">
         <is>
-          <t>persona.ttl (→ PersonOntology on promotion)</t>
+          <t>PersonOntology</t>
         </is>
       </c>
       <c r="F45" s="34" t="inlineStr"/>
       <c r="G45" s="35" t="inlineStr">
         <is>
-          <t>Minted</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="H45" s="34" t="inlineStr">
@@ -4129,14 +4102,12 @@
           <t>PersonOntology</t>
         </is>
       </c>
-      <c r="K45" s="35" t="inlineStr">
-        <is>
-          <t>2026-03-17</t>
-        </is>
+      <c r="K45" s="51" t="n">
+        <v>46214</v>
       </c>
       <c r="L45" s="33" t="inlineStr">
         <is>
-          <t>skos:exactMatch cco:ont00000797</t>
+          <t>skos:exactMatch cco:ont00000797; Promoted to PersonOntology 2026-07-11 (committed to Main); Option B: closeMatch (not exactMatch) to CCO colors</t>
         </is>
       </c>
       <c r="M45" s="34" t="inlineStr">
@@ -4240,38 +4211,38 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="46" t="inlineStr">
+      <c r="A47" s="48" t="inlineStr">
         <is>
           <t>ent00000046</t>
         </is>
       </c>
-      <c r="B47" s="46" t="inlineStr">
+      <c r="B47" s="48" t="inlineStr">
         <is>
           <t>https://purl.org/cco/ent00000046</t>
         </is>
       </c>
-      <c r="C47" s="47" t="inlineStr">
+      <c r="C47" s="49" t="inlineStr">
         <is>
           <t>Birthdate</t>
         </is>
       </c>
-      <c r="D47" s="47" t="inlineStr">
+      <c r="D47" s="49" t="inlineStr">
         <is>
           <t>owl:Class</t>
         </is>
       </c>
-      <c r="E47" s="47" t="inlineStr">
+      <c r="E47" s="49" t="inlineStr">
         <is>
           <t>PersonOntology</t>
         </is>
       </c>
-      <c r="F47" s="46" t="inlineStr"/>
-      <c r="G47" s="47" t="inlineStr">
+      <c r="F47" s="48" t="inlineStr"/>
+      <c r="G47" s="49" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="H47" s="46" t="inlineStr">
+      <c r="H47" s="48" t="inlineStr">
         <is>
           <t>https://purl.org/cco/ont00001340  # Calendar Date Identifier</t>
         </is>
@@ -4281,115 +4252,113 @@
           <t>A Calendar Date Identifier that designates the date on which a Person was born.</t>
         </is>
       </c>
-      <c r="J47" s="47" t="inlineStr">
+      <c r="J47" s="49" t="inlineStr">
         <is>
           <t>PersonOntology</t>
         </is>
       </c>
-      <c r="K47" s="47" t="inlineStr">
+      <c r="K47" s="50" t="n">
+        <v>46126</v>
+      </c>
+      <c r="L47" s="4" t="inlineStr">
+        <is>
+          <t>RFC 9553 §2.8.1; corrects Claude Code's wrong parent (Quality)</t>
+        </is>
+      </c>
+      <c r="M47" s="48" t="inlineStr">
+        <is>
+          <t>https://purl.org/cco/ent00000046</t>
+        </is>
+      </c>
+      <c r="N47" s="48" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O47" s="4" t="inlineStr">
+        <is>
+          <t>Register new ent PURL → ontology file</t>
+        </is>
+      </c>
+      <c r="P47" s="48" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/ethical-freelancing/EFO/main/ontology/domains/PersonOntology.ttl</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="48" t="inlineStr">
+        <is>
+          <t>ent00000047</t>
+        </is>
+      </c>
+      <c r="B48" s="48" t="inlineStr">
+        <is>
+          <t>https://purl.org/cco/ent00000047</t>
+        </is>
+      </c>
+      <c r="C48" s="49" t="inlineStr">
+        <is>
+          <t>Organization Name</t>
+        </is>
+      </c>
+      <c r="D48" s="49" t="inlineStr">
+        <is>
+          <t>owl:Class</t>
+        </is>
+      </c>
+      <c r="E48" s="49" t="inlineStr">
+        <is>
+          <t>StagingOntology</t>
+        </is>
+      </c>
+      <c r="F48" s="48" t="inlineStr"/>
+      <c r="G48" s="49" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="H48" s="48" t="inlineStr">
+        <is>
+          <t>https://purl.org/cco/ont00000003  # Designative Name</t>
+        </is>
+      </c>
+      <c r="I48" s="4" t="inlineStr">
+        <is>
+          <t>A Designative Name that designates an Organization a Person is affiliated with.</t>
+        </is>
+      </c>
+      <c r="J48" s="49" t="inlineStr">
+        <is>
+          <t>Future Organization Ontology</t>
+        </is>
+      </c>
+      <c r="K48" s="49" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
       </c>
-      <c r="L47" s="4" t="inlineStr">
-        <is>
-          <t>RFC 9553 §2.8.1; corrects Claude Code's wrong parent (Quality)</t>
-        </is>
-      </c>
-      <c r="M47" s="46" t="inlineStr">
-        <is>
-          <t>https://purl.org/cco/ent00000046</t>
-        </is>
-      </c>
-      <c r="N47" s="46" t="inlineStr">
+      <c r="L48" s="4" t="inlineStr">
+        <is>
+          <t>RFC 9553 §2.2.2; Placed in StagingOntology 2026-07-09 per Mee alignment; migration target undecided</t>
+        </is>
+      </c>
+      <c r="M48" s="48" t="inlineStr">
+        <is>
+          <t>https://purl.org/cco/ent00000047</t>
+        </is>
+      </c>
+      <c r="N48" s="48" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="O47" s="4" t="inlineStr">
+      <c r="O48" s="4" t="inlineStr">
         <is>
           <t>Register new ent PURL → ontology file</t>
         </is>
       </c>
-      <c r="P47" s="46" t="inlineStr">
-        <is>
-          <t>https://raw.githubusercontent.com/ethical-freelancing/EFO/main/ontology/domains/PersonOntology.ttl</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="46" t="inlineStr">
-        <is>
-          <t>ent00000047</t>
-        </is>
-      </c>
-      <c r="B48" s="46" t="inlineStr">
-        <is>
-          <t>https://purl.org/cco/ent00000047</t>
-        </is>
-      </c>
-      <c r="C48" s="47" t="inlineStr">
-        <is>
-          <t>Organization Name</t>
-        </is>
-      </c>
-      <c r="D48" s="47" t="inlineStr">
-        <is>
-          <t>owl:Class</t>
-        </is>
-      </c>
-      <c r="E48" s="47" t="inlineStr">
-        <is>
-          <t>PersonOntology</t>
-        </is>
-      </c>
-      <c r="F48" s="46" t="inlineStr"/>
-      <c r="G48" s="47" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="H48" s="46" t="inlineStr">
-        <is>
-          <t>https://purl.org/cco/ont00000003  # Designative Name</t>
-        </is>
-      </c>
-      <c r="I48" s="4" t="inlineStr">
-        <is>
-          <t>A Designative Name that designates an Organization a Person is affiliated with.</t>
-        </is>
-      </c>
-      <c r="J48" s="47" t="inlineStr">
-        <is>
-          <t>PersonOntology</t>
-        </is>
-      </c>
-      <c r="K48" s="47" t="inlineStr">
-        <is>
-          <t>2026-03-17</t>
-        </is>
-      </c>
-      <c r="L48" s="4" t="inlineStr">
-        <is>
-          <t>RFC 9553 §2.2.2</t>
-        </is>
-      </c>
-      <c r="M48" s="46" t="inlineStr">
-        <is>
-          <t>https://purl.org/cco/ent00000047</t>
-        </is>
-      </c>
-      <c r="N48" s="46" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O48" s="4" t="inlineStr">
-        <is>
-          <t>Register new ent PURL → ontology file</t>
-        </is>
-      </c>
-      <c r="P48" s="46" t="inlineStr">
+      <c r="P48" s="48" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/ethical-freelancing/EFO/main/ontology/domains/PersonOntology.ttl</t>
         </is>
@@ -4424,7 +4393,7 @@
       <c r="F49" s="44" t="inlineStr"/>
       <c r="G49" s="45" t="inlineStr">
         <is>
-          <t>Proposed</t>
+          <t>Removed</t>
         </is>
       </c>
       <c r="H49" s="44" t="inlineStr">
@@ -4439,7 +4408,7 @@
       </c>
       <c r="J49" s="45" t="inlineStr">
         <is>
-          <t>PersonOntology or Contact WG 2026-Q3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K49" s="45" t="inlineStr">
@@ -4449,7 +4418,7 @@
       </c>
       <c r="L49" s="10" t="inlineStr">
         <is>
-          <t>RFC 9553 §2.8.3; corrects Claude Code's wrong parent (Desig. Name)</t>
+          <t>RFC 9553 §2.8.3; corrects Claude Code's wrong parent (Desig. Name); Removed 2026-07-09: no consumer; generic Descriptive ICE (ont00000853) sufficient</t>
         </is>
       </c>
       <c r="M49" s="44" t="inlineStr">
@@ -4917,7 +4886,7 @@
       </c>
       <c r="L55" s="10" t="inlineStr">
         <is>
-          <t>Parent fixed from TimeOfDayIdentifier to CalendarDateIdentifier</t>
+          <t>Parent fixed from TimeOfDayIdentifier to CalendarDateIdentifier; Superseded 2026-07-13 by ent00000070 (has expiration date) property pattern; retained pending Paul data migration, then deprecate</t>
         </is>
       </c>
       <c r="M55" s="44" t="inlineStr">
@@ -4988,110 +4957,108 @@
           <t>CyberOntology (P3195.1.1) 2026-Q3</t>
         </is>
       </c>
-      <c r="K56" s="45" t="inlineStr">
+      <c r="K56" s="52" t="n">
+        <v>46212</v>
+      </c>
+      <c r="L56" s="10" t="inlineStr">
+        <is>
+          <t>Superclass of TelephoneNumber and EmailAddress; migrated from Orphan</t>
+        </is>
+      </c>
+      <c r="M56" s="44" t="inlineStr">
+        <is>
+          <t>https://purl.org/cco/ent00000055</t>
+        </is>
+      </c>
+      <c r="N56" s="44" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O56" s="10" t="inlineStr">
+        <is>
+          <t>Register new ent PURL → ontology file</t>
+        </is>
+      </c>
+      <c r="P56" s="44" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/ethical-freelancing/EFO/main/ontology/domains/StagingOntology.ttl</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="48" t="inlineStr">
+        <is>
+          <t>ent00000056</t>
+        </is>
+      </c>
+      <c r="B57" s="48" t="inlineStr">
+        <is>
+          <t>https://purl.org/cco/ent00000056</t>
+        </is>
+      </c>
+      <c r="C57" s="49" t="inlineStr">
+        <is>
+          <t>Postal Zone</t>
+        </is>
+      </c>
+      <c r="D57" s="49" t="inlineStr">
+        <is>
+          <t>owl:Class</t>
+        </is>
+      </c>
+      <c r="E57" s="49" t="inlineStr">
+        <is>
+          <t>AddressOntology</t>
+        </is>
+      </c>
+      <c r="F57" s="48" t="inlineStr"/>
+      <c r="G57" s="49" t="inlineStr">
+        <is>
+          <t>Removed</t>
+        </is>
+      </c>
+      <c r="H57" s="48" t="inlineStr">
+        <is>
+          <t>https://purl.org/cco/ont00000460  # Local Administrative Region</t>
+        </is>
+      </c>
+      <c r="I57" s="4" t="inlineStr">
+        <is>
+          <t>A Local Administrative Region delimiting delivery points within a postal system.</t>
+        </is>
+      </c>
+      <c r="J57" s="49" t="inlineStr">
+        <is>
+          <t>PostalAddressOntology</t>
+        </is>
+      </c>
+      <c r="K57" s="49" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
       </c>
-      <c r="L56" s="10" t="inlineStr">
-        <is>
-          <t>Superclass of TelephoneNumber and EmailAddress; migrated from Orphan</t>
-        </is>
-      </c>
-      <c r="M56" s="44" t="inlineStr">
-        <is>
-          <t>https://purl.org/cco/ent00000055</t>
-        </is>
-      </c>
-      <c r="N56" s="44" t="inlineStr">
+      <c r="L57" s="4" t="inlineStr">
+        <is>
+          <t>Geographic region designated by a PostalCode; migrated from Orphan | Term not present in committed AddressOntology.ttl as of 2026-08-05; marked Removed per registry-audit finding.</t>
+        </is>
+      </c>
+      <c r="M57" s="48" t="inlineStr">
+        <is>
+          <t>https://purl.org/cco/ent00000056</t>
+        </is>
+      </c>
+      <c r="N57" s="48" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="O56" s="10" t="inlineStr">
+      <c r="O57" s="4" t="inlineStr">
         <is>
           <t>Register new ent PURL → ontology file</t>
         </is>
       </c>
-      <c r="P56" s="44" t="inlineStr">
-        <is>
-          <t>https://raw.githubusercontent.com/ethical-freelancing/EFO/main/ontology/domains/StagingOntology.ttl</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="46" t="inlineStr">
-        <is>
-          <t>ent00000056</t>
-        </is>
-      </c>
-      <c r="B57" s="46" t="inlineStr">
-        <is>
-          <t>https://purl.org/cco/ent00000056</t>
-        </is>
-      </c>
-      <c r="C57" s="47" t="inlineStr">
-        <is>
-          <t>Postal Zone</t>
-        </is>
-      </c>
-      <c r="D57" s="47" t="inlineStr">
-        <is>
-          <t>owl:Class</t>
-        </is>
-      </c>
-      <c r="E57" s="47" t="inlineStr">
-        <is>
-          <t>PostalAddressOntology</t>
-        </is>
-      </c>
-      <c r="F57" s="46" t="inlineStr"/>
-      <c r="G57" s="47" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="H57" s="46" t="inlineStr">
-        <is>
-          <t>https://purl.org/cco/ont00000460  # Local Administrative Region</t>
-        </is>
-      </c>
-      <c r="I57" s="4" t="inlineStr">
-        <is>
-          <t>A Local Administrative Region delimiting delivery points within a postal system.</t>
-        </is>
-      </c>
-      <c r="J57" s="47" t="inlineStr">
-        <is>
-          <t>PostalAddressOntology</t>
-        </is>
-      </c>
-      <c r="K57" s="47" t="inlineStr">
-        <is>
-          <t>2026-03-17</t>
-        </is>
-      </c>
-      <c r="L57" s="4" t="inlineStr">
-        <is>
-          <t>Geographic region designated by a PostalCode; migrated from Orphan</t>
-        </is>
-      </c>
-      <c r="M57" s="46" t="inlineStr">
-        <is>
-          <t>https://purl.org/cco/ent00000056</t>
-        </is>
-      </c>
-      <c r="N57" s="46" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O57" s="4" t="inlineStr">
-        <is>
-          <t>Register new ent PURL → ontology file</t>
-        </is>
-      </c>
-      <c r="P57" s="46" t="inlineStr">
+      <c r="P57" s="48" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/ethical-freelancing/EFO/main/ontology/domains/PostalAddressOntology.ttl</t>
         </is>
@@ -5144,10 +5111,8 @@
           <t>PersonOntology</t>
         </is>
       </c>
-      <c r="K58" s="49" t="inlineStr">
-        <is>
-          <t>2026-03-17</t>
-        </is>
+      <c r="K58" s="50" t="n">
+        <v>46143</v>
       </c>
       <c r="L58" s="4" t="inlineStr">
         <is>
@@ -5222,10 +5187,8 @@
           <t>PersonOntology</t>
         </is>
       </c>
-      <c r="K59" s="49" t="inlineStr">
-        <is>
-          <t>2026-03-17</t>
-        </is>
+      <c r="K59" s="50" t="n">
+        <v>46143</v>
       </c>
       <c r="L59" s="4" t="inlineStr">
         <is>
@@ -5276,7 +5239,7 @@
       </c>
       <c r="E60" s="49" t="inlineStr">
         <is>
-          <t>PostalAddressOntology</t>
+          <t>AddressOntology</t>
         </is>
       </c>
       <c r="F60" s="48" t="inlineStr"/>
@@ -5287,7 +5250,7 @@
       </c>
       <c r="H60" s="48" t="inlineStr">
         <is>
-          <t>https://purl.org/cco/ont00000077  # Code Identifier</t>
+          <t>cco:ent00000312</t>
         </is>
       </c>
       <c r="I60" s="4" t="inlineStr">
@@ -5300,10 +5263,8 @@
           <t>PostalAddressOntology</t>
         </is>
       </c>
-      <c r="K60" s="49" t="inlineStr">
-        <is>
-          <t>2026-03-17</t>
-        </is>
+      <c r="K60" s="50" t="n">
+        <v>46209</v>
       </c>
       <c r="L60" s="4" t="inlineStr">
         <is>
@@ -5334,27 +5295,27 @@
     <row r="61">
       <c r="A61" s="48" t="inlineStr">
         <is>
-          <t>ent00000060</t>
+          <t>ent00000061</t>
         </is>
       </c>
       <c r="B61" s="48" t="inlineStr">
         <is>
-          <t>https://purl.org/cco/ent00000060</t>
+          <t>https://purl.org/cco/ent00000061</t>
         </is>
       </c>
       <c r="C61" s="49" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>has birthdate</t>
         </is>
       </c>
       <c r="D61" s="49" t="inlineStr">
         <is>
-          <t>owl:NamedIndividual</t>
+          <t>owl:ObjectProperty</t>
         </is>
       </c>
       <c r="E61" s="49" t="inlineStr">
         <is>
-          <t>PostalAddressOntology</t>
+          <t>PersonOntology</t>
         </is>
       </c>
       <c r="F61" s="48" t="inlineStr"/>
@@ -5365,47 +5326,1307 @@
       </c>
       <c r="H61" s="48" t="inlineStr">
         <is>
-          <t>https://purl.org/cco/ent00000059  # Country Code</t>
+          <t>https://purl.org/cco/ont00001262  # domain Person / range Birthdate</t>
         </is>
       </c>
       <c r="I61" s="4" t="inlineStr">
         <is>
-          <t>ISO 3166-1 code designating the United States of America. altLabels: USA, 840.</t>
+          <t>Each instance of Person has an instance of Birthdate.</t>
         </is>
       </c>
       <c r="J61" s="49" t="inlineStr">
         <is>
+          <t>PersonOntology</t>
+        </is>
+      </c>
+      <c r="K61" s="54" t="n">
+        <v>46130</v>
+      </c>
+      <c r="L61" s="4" t="inlineStr">
+        <is>
+          <t>Added in July 6 rebuild</t>
+        </is>
+      </c>
+      <c r="M61" s="48" t="inlineStr">
+        <is>
+          <t>https://purl.org/cco/ent00000060</t>
+        </is>
+      </c>
+      <c r="N61" s="48" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O61" s="4" t="inlineStr">
+        <is>
+          <t>Register new ent PURL → ontology file</t>
+        </is>
+      </c>
+      <c r="P61" s="48" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/ethical-freelancing/EFO/main/ontology/domains/PostalAddressOntology.ttl</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>ent00000062</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>https://purl.org/cco/ent00000062</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Person Identifier</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>owl:Class</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>PersonOntology</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>https://purl.org/cco/ont00000649  # non-Name Identifier</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>A non-Name Identifier for a person.</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>PersonOntology</t>
+        </is>
+      </c>
+      <c r="K62" s="55" t="n">
+        <v>46132</v>
+      </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>Renamed from has city name value</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>ent00000063</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>https://purl.org/cco/ent00000063</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Maroon Eye Color</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>owl:Class</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>PersonOntology</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>https://purl.org/cco/ent00000037</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>An Eye Color that appears maroon.</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>PersonOntology</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>closeMatch CCO Maroon (ont00000913); minted 2026-07-11 for AAMVA MAR coverage</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>ent00000064</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>https://purl.org/cco/ent00000064</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Pink/Red Eye Color</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>owl:Class</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>PersonOntology</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>https://purl.org/cco/ent00000037</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>An Eye Color that appears pink or light red due to lack of pigmentation.</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>PersonOntology</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>closeMatch CCO Red (ont00001277); minted 2026-07-11 for AAMVA PNK/albinism coverage</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>ent00000065</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>https://purl.org/cco/ent00000065</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Drivers License Number</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>owl:Class</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>PersonOntology</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>https://purl.org/cco/ent00000062  # Person Identifier</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>A Person Identifier issued to a person by a driver-licensing authority.</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>PersonOntology</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>Promoted from Mee persona:DriversLicenseNumber 2026-07-11; sibling of SSN under Person Identifier</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>ent00000066</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>https://purl.org/cco/ent00000066</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Passport Number</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>owl:Class</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>PersonOntology</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>https://purl.org/cco/ent00000062  # Person Identifier</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>A Person Identifier issued to a person by a passport-issuing authority.</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>PersonOntology</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>Promoted from Mee persona:PassportNumber 2026-07-11; sibling of SSN under Person Identifier</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>ent00000067</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>https://purl.org/cco/ent00000067</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Place of Birth</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>owl:Class</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>PersonOntology</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>https://purl.org/cco/ont00000686  # Designative Information Content Entity</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>A Designative ICE that designates the civil jurisdiction in which a person's birth was registered, as recorded on an identity document (may differ from geographic birth location).</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>PersonOntology</t>
+        </is>
+      </c>
+      <c r="K67" s="53" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>Promoted from Mee persona:PlaceOfBirth 2026-07-11; Option A (string designator, registration-jurisdiction semantics)</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>ent00000068</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>https://purl.org/cco/ent00000068</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Issuing Jurisdiction</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>owl:Class</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>PersonOntology</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>https://purl.org/cco/ont00000686  # Designative Information Content Entity</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>A Designative ICE designating the governmental authority that issued an identity document, at any level (national/state/agency/municipal), as recorded on the document. Not a postal address component.</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>PersonOntology</t>
+        </is>
+      </c>
+      <c r="K68" s="53" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>Promoted from Mee persona:IssuingJurisdiction AND persona:IssuingCountry 2026-07-11 (both collapse to this level-agnostic term); string designator, issuer-authority semantics</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>ent00000069</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>https://purl.org/cco/ent00000069</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>has issue date</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>owl:ObjectProperty</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>StagingOntology</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>https://purl.org/cco/ont00001879 (subPropertyOf 'designated by'); range ont00001340 (Calendar Date Identifier)</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>Relates an issued thing to the Calendar Date Identifier designating the date on which it was issued.</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>StagingOntology</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>Option B (role-as-relation, not subclass); promoted from Mee persona:IssueDate 2026-07-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>ent00000070</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>https://purl.org/cco/ent00000070</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>has expiration date</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>owl:ObjectProperty</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>StagingOntology</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>https://purl.org/cco/ont00001879 (subPropertyOf 'designated by'); range ont00001340 (Calendar Date Identifier)</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>Relates a thing with a validity period to the Calendar Date Identifier designating the date after which it is no longer valid.</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>StagingOntology</t>
+        </is>
+      </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>Option B (role-as-relation); SUPERSEDES ent00000054 ExpirationDateIdentifier subclass; migrate Paul's data in gov-ID PR bundle</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>ent00000071</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>https://purl.org/cco/ent00000071</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Checking Account Number</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>owl:Class</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>StagingOntology</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>https://purl.org/cco/ont00000077  # Code Identifier</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>A Code Identifier that designates a checking account within a financial institution's system of record.</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>StagingOntology</t>
+        </is>
+      </c>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t>DL-011 (DP-1 Option A); promoted from Mee persona:CheckingAccountNumber; FinanceCluster Architecture v0.1 §5</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>ent00000072</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>https://purl.org/cco/ent00000072</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Routing Number</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>owl:Class</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>StagingOntology</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>https://purl.org/cco/ont00000077  # Code Identifier</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>A Code Identifier that designates a financial institution within a payment clearing network for routing payments.</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>StagingOntology</t>
+        </is>
+      </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="L72" t="inlineStr">
+        <is>
+          <t>DL-011 (DP-1 Option A); institution-level identifier — see FinanceCluster Architecture v0.1 §5.2 for pre-specified refactor trigger (Financial Institution Identifier intermediate on 2nd institution-level identifier); promoted from Mee persona:RoutingNumber</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>ent00000073</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>https://purl.org/cco/ent00000073</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>has payment card</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>owl:ObjectProperty</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>StagingOntology</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>persona:hasPaymentCard (Mee — migrates at promotion PR)</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>(bare ObjectProperty; domain cco:ont00001017 Agent, range cco:ent00000049 Payment Card)</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>Relates an Agent to a Payment Card the Agent has and is authorized to use.</t>
+        </is>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>StagingOntology</t>
+        </is>
+      </c>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="L73" t="inlineStr">
+        <is>
+          <t>DL-010; promoted from Mee persona:hasPaymentCard; closes Wave 2.5; date-annotation omitted from stanza per deferred date-drift cleanup</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>ent00000310</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>https://purl.org/cco/ent00000068</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Address</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>owl:Class</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>AddressOntology</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>cco:ont00000958</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>An ICE that identifies a physical location of a person, facility or organization for the purpose of communication or service.</t>
+        </is>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>PersonOntology</t>
+        </is>
+      </c>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="L74" t="inlineStr">
+        <is>
+          <t>Added to registry retroactively 2026-08 (registry-audit finding); committed in file since 2026-06-15, not previously registered.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>ent00000312</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>https://purl.org/cco/ent00000069</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Address Component</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>owl:Class</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>AddressOntology</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>cco:ont00000958</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>An ICE that is part of an address and provides a specific piece of information needed to locate or identify the address target.</t>
+        </is>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>StagingOntology</t>
+        </is>
+      </c>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="L75" t="inlineStr">
+        <is>
+          <t>Added to registry retroactively 2026-08 (registry-audit finding); parent of Country Name/Code and other address components.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>ent00000316</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>https://purl.org/cco/ent00000070</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>has address component</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>owl:ObjectProperty</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>AddressOntology</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>domain cco:ent00000310 / range cco:ent00000312</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>Connects an Address instance to an AddressComponent instance that is part of that address. Inverse of ent00000317.</t>
+        </is>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>StagingOntology</t>
+        </is>
+      </c>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="L76" t="inlineStr">
+        <is>
+          <t>Added to registry retroactively 2026-08 (registry-audit finding).</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>ent00000317</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>https://purl.org/cco/ent00000071</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>is address component of</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>owl:ObjectProperty</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>AddressOntology</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>domain cco:ent00000312 / range cco:ent00000310</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>Connects an AddressComponent instance to the Address it is part of. Inverse of ent00000316.</t>
+        </is>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>StagingOntology</t>
+        </is>
+      </c>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="L77" t="inlineStr">
+        <is>
+          <t>Added to registry retroactively 2026-08 (registry-audit finding). Definition text in file has a drafting error (self-cites ent00000316; states wrong direction) — flagged for Jim to fix in Protégé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>ent00000318</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>https://purl.org/cco/ent00000318</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>has street address value</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>owl:DatatypeProperty</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>AddressOntology</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>cco:ent00000011</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>Datatype property for Street Address value</t>
+        </is>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
           <t>PostalAddressOntology</t>
         </is>
       </c>
-      <c r="K61" s="49" t="inlineStr">
-        <is>
-          <t>2026-03-17</t>
-        </is>
-      </c>
-      <c r="L61" s="4" t="inlineStr">
-        <is>
-          <t>First Named Individual in registry — demonstrates ent scheme covers instances too</t>
-        </is>
-      </c>
-      <c r="M61" s="48" t="inlineStr">
+      <c r="K78" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="L78" t="inlineStr">
+        <is>
+          <t>Added in July 6 rebuild</t>
+        </is>
+      </c>
+      <c r="M78" t="inlineStr">
         <is>
           <t>https://purl.org/cco/ent00000060</t>
         </is>
       </c>
-      <c r="N61" s="48" t="inlineStr">
+      <c r="N78" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="O61" s="4" t="inlineStr">
+      <c r="O78" t="inlineStr">
         <is>
           <t>Register new ent PURL → ontology file</t>
         </is>
       </c>
-      <c r="P61" s="48" t="inlineStr">
+      <c r="P78" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/ethical-freelancing/EFO/main/ontology/domains/PostalAddressOntology.ttl</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>ent00000319</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>https://purl.org/cco/ent00000319</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>has city value</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>owl:DatatypeProperty</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>AddressOntology</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>persona:hasPaymentCard (Mee — migrates at promotion PR)</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>cco:ent00000012</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>Datatype property for City value</t>
+        </is>
+      </c>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>StagingOntology</t>
+        </is>
+      </c>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="L79" t="inlineStr">
+        <is>
+          <t>Renamed from has city name value</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>ent00000320</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>https://purl.org/cco/ent00000320</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>has state value</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>owl:DatatypeProperty</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>AddressOntology</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>cco:ent00000013</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>Datatype property for State value</t>
+        </is>
+      </c>
+      <c r="K80" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="L80" t="inlineStr">
+        <is>
+          <t>Renamed from has state name value</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>ent00000321</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>https://purl.org/cco/ent00000321</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>has postal code value</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>owl:DatatypeProperty</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>AddressOntology</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>cco:ent00000015</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>Datatype property for Postal Code value</t>
+        </is>
+      </c>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="L81" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>ent00000322</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>https://purl.org/cco/ent00000322</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>has country code value</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>owl:DatatypeProperty</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>AddressOntology</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>cco:ent00000059</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>Datatype property for Country Code value</t>
+        </is>
+      </c>
+      <c r="K82" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="L82" t="inlineStr">
+        <is>
+          <t>NEW - FunctionalProperty</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>ent00000323</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>https://purl.org/cco/ent00000323</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>has country name value</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>owl:DatatypeProperty</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>AddressOntology</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>cco:ent00000014</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>Datatype property for Country Name value</t>
+        </is>
+      </c>
+      <c r="K83" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="L83" t="inlineStr">
+        <is>
+          <t>NEW</t>
         </is>
       </c>
     </row>
@@ -5624,7 +6845,6 @@
         </is>
       </c>
     </row>
-    <row r="21"/>
     <row r="22">
       <c r="A22" s="36" t="inlineStr"/>
       <c r="B22" s="17" t="inlineStr"/>

</xml_diff>